<commit_message>
Atualização das emendas federais (23/09/2026 11:30)
</commit_message>
<xml_diff>
--- a/upload/dados_gerais_emendas.xlsx
+++ b/upload/dados_gerais_emendas.xlsx
@@ -1128,7 +1128,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">	Transferência Especial para aquisição de viaturas (uma caracterizada e uma descaracterizada), computadores, aeronave remotamente pilotada (RPA - drone), impressoras multifuncionais, switch, Plotter, computadores e notebooks para a 5ª Delegacia Regional de Polícia Civil de Viçosa/MG.</t>
+          <t>Transferência Especial para aquisição de viaturas (uma caracterizada e uma descaracterizada), computadores, aeronave remotamente pilotada (RPA - drone), impressoras multifuncionais, switch, Plotter, computadores e notebooks para a 5ª Delegacia Regional de Polícia Civil de Viçosa/MG.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1258,9 +1258,8 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fortalecimento da Polícia Militar de Minas Gerais por meio de aquisição de motocicletas para os seguintes Municípios: 42º BPM- Curvelo/MG; 13ª Cia Ind - Brasília De Minas/MG; 15º BPM - Carmo Do
-Paranaíba/MG; 31º BPM - Congonhas/MG; 7º BPM - Lagoa Da Prata/MG; 46º BPM - Patrocínio/MG; 31º BPM - Ouro Branco/MG; 28º BPM - Unaí/MG.
-</t>
+          <t>Fortalecimento da Polícia Militar de Minas Gerais por meio de aquisição de motocicletas para os seguintes Municípios: 42º BPM- Curvelo/MG; 13ª Cia Ind - Brasília De Minas/MG; 15º BPM - Carmo Do
+Paranaíba/MG; 31º BPM - Congonhas/MG; 7º BPM - Lagoa Da Prata/MG; 46º BPM - Patrocínio/MG; 31º BPM - Ouro Branco/MG; 28º BPM - Unaí/MG.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -4403,7 +4402,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t xml:space="preserve">918013/2021 </t>
+          <t>918013/2021</t>
         </is>
       </c>
       <c r="I62" t="n">
@@ -4468,7 +4467,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t xml:space="preserve">918015/2021 </t>
+          <t>918015/2021</t>
         </is>
       </c>
       <c r="I63" t="n">
@@ -6341,7 +6340,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t xml:space="preserve">916827/2021 </t>
+          <t>916827/2021</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -6406,7 +6405,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t xml:space="preserve">911951/2021 </t>
+          <t>911951/2021</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -9735,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t xml:space="preserve">1415/2022 </t>
+          <t>1415/2022</t>
         </is>
       </c>
       <c r="I146" t="n">
@@ -9991,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t xml:space="preserve">1684/2022 </t>
+          <t>1684/2022</t>
         </is>
       </c>
       <c r="I150" t="n">
@@ -10387,7 +10386,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Recurso destinado para estruturação de unidade do CBMMG em Juiz de Fora</t>
+          <t>Recurso destinado para estruturação de unidade do CBMMG em Juiz de Fora</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
@@ -10452,8 +10451,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transferência Especial para  custeio de ações de Proteção Animal
-</t>
+          <t>Transferência Especial para  custeio de ações de Proteção Animal</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
@@ -10648,7 +10646,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Reforma da edificação do Pelotão de Emergências Ambientais e Desastres (PEMAD) e construção do Centro de Capacitação Permanente “D.PEDRO II” (CCP) – ambos localizados em Juiz de Fora.</t>
+          <t>Reforma da edificação do Pelotão de Emergências Ambientais e Desastres (PEMAD) e construção do Centro de Capacitação Permanente “D.PEDRO II” (CCP) – ambos localizados em Juiz de Fora.</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -12064,7 +12062,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t xml:space="preserve">936054/2022 </t>
+          <t>936054/2022</t>
         </is>
       </c>
       <c r="I182" t="n">
@@ -12403,8 +12401,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transferência Especial para aquisição de computadores para a Escola Estadual José Ermírio de Morais em Três Marias
-</t>
+          <t>Transferência Especial para aquisição de computadores para a Escola Estadual José Ermírio de Morais em Três Marias</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
@@ -13170,7 +13167,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t xml:space="preserve">927358/2022 </t>
+          <t>927358/2022</t>
         </is>
       </c>
       <c r="I199" t="n">
@@ -13249,8 +13246,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transferência Especial para Obra de Ampliação do Posto Avançado do CBMMG no município de Boa Esperança/MG.
-</t>
+          <t>Transferência Especial para Obra de Ampliação do Posto Avançado do CBMMG no município de Boa Esperança/MG.</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -13705,8 +13701,7 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aquisição de equipamentos para o Presídio de Itajubá/MG.
-</t>
+          <t>Aquisição de equipamentos para o Presídio de Itajubá/MG.</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
@@ -13836,8 +13831,7 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transferência Especial para aquisição de Patrulha Agrícola Mecanizada para a Empresa de Assistência Técnica e Extensão Rural de Minas Gerais – Emater – Unidade de Alvinópolis. A aquisição tem por objetivo maior eficiência produtiva, desenvolvimento agrícola, melhoria de renda e da qualidade de vida dos agricultores familiares, para uso na Associação de Desenvolvimento Comunitário
-</t>
+          <t>Transferência Especial para aquisição de Patrulha Agrícola Mecanizada para a Empresa de Assistência Técnica e Extensão Rural de Minas Gerais – Emater – Unidade de Alvinópolis. A aquisição tem por objetivo maior eficiência produtiva, desenvolvimento agrícola, melhoria de renda e da qualidade de vida dos agricultores familiares, para uso na Associação de Desenvolvimento Comunitário</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
@@ -14812,8 +14806,7 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Execução de obras na Academia de Bombeiros Militar em Belo Horizonte/MG
-</t>
+          <t>Execução de obras na Academia de Bombeiros Militar em Belo Horizonte/MG</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
@@ -18022,8 +18015,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reforma/Construção/Ampliação da Delegacia Especializada de Atendimento à Mulher de Teófilo Otoni/MG.
-</t>
+          <t>Reforma/Construção/Ampliação da Delegacia Especializada de Atendimento à Mulher de Teófilo Otoni/MG.</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -18153,8 +18145,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serviços de reforma e adaptação de bens imóveis em unidades da PCMG.
-</t>
+          <t>Serviços de reforma e adaptação de bens imóveis em unidades da PCMG.</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
@@ -18219,8 +18210,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transferência Especial para Estruturação do Corpo de Bombeiros de Contagem e Passos / MG.
-</t>
+          <t>Transferência Especial para Estruturação do Corpo de Bombeiros de Contagem e Passos / MG.</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -19130,7 +19120,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aquisição de aeronaves remotamente pilotadas, equipamentos de uso policial, equipamentos de informática, aquisição de viaturas, aquisição de mobiliário, utensílios e equipamento de uso administrativo. </t>
+          <t>Aquisição de aeronaves remotamente pilotadas, equipamentos de uso policial, equipamentos de informática, aquisição de viaturas, aquisição de mobiliário, utensílios e equipamento de uso administrativo.</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
@@ -19585,8 +19575,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-Aquisição de Aquisição de Aeronave Remotamente Pilotada (DRONE) para a PCMG.</t>
+          <t>Aquisição de Aquisição de Aeronave Remotamente Pilotada (DRONE) para a PCMG.</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">

</xml_diff>